<commit_message>
Mapa: OSM France en vez de tile.openstreetmap.org (bloquea peticiones sin Referer, p. ej. la copia HTML); ejemplo Japón actualizado
</commit_message>
<xml_diff>
--- a/ejemplos/japon-2026-hitos.xlsx
+++ b/ejemplos/japon-2026-hitos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L347"/>
+  <dimension ref="A1:L351"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8936,6 +8936,106 @@
         </is>
       </c>
     </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>Ōya History Museum</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Cantera industrial de piedra Ōya (1919–1986)</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Utsunomiya</t>
+        </is>
+      </c>
+      <c r="E348" t="n">
+        <v>1979</v>
+      </c>
+      <c r="L348" t="inlineStr">
+        <is>
+          <t>S · Antigua cantera subterránea: una arquitectura del vacío, la escala y la temperatura. No es obra de autor, pero espacialmente es brutal</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>Stone Plaza</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Kengo Kuma</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Nasu</t>
+        </is>
+      </c>
+      <c r="E349" t="n">
+        <v>2000</v>
+      </c>
+      <c r="L349" t="inlineStr">
+        <is>
+          <t>A+/S− · Tres almacenes de piedra transformados mediante muros porosos, lamas pétreas, agua y luz. Encaja extraordinariamente bien antes de Ishigami (Water Garden)</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>Nasu History Museum</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Kengo Kuma</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Nasu</t>
+        </is>
+      </c>
+      <c r="E350" t="n">
+        <v>2000</v>
+      </c>
+      <c r="L350" t="inlineStr">
+        <is>
+          <t>A · Pequeño, transparente y casi desmaterializado; a unos diez minutos andando de Stone Plaza</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>Suite Villas (Art Biotop Nasu)</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Shigeru Ban</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Nasu</t>
+        </is>
+      </c>
+      <c r="E351" t="n">
+        <v>2018</v>
+      </c>
+      <c r="L351" t="inlineStr">
+        <is>
+          <t>A+ si permiten visita [R] · En el propio complejo de Water Garden: catorce villas de madera con estructura de grandes cerchas y piedra excavada del solar. Preguntar si permiten visita</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sesiones de edición, diario de cambios con deshacer y página de administración oculta
Cada cambio (curado, edición, borrado, plantillas, fotos, viajes) queda anotado en
`changes` con lo necesario para deshacerlo; la sesión de un navegador se abre con su
primer cambio y se cierra tras 1 h sin actividad. Página #/admin (triple clic en el
pie, contraseña ARCHTRIP_ADMIN_PASSWORD, "admin" por defecto): sesiones con nombre,
deshacer un cambio o toda la sesión, historial de un hito, copias de seguridad
(crear, descargar, volcado SQL, restaurar con copia previa). Los archivos de fotos
borradas se conservan para poder restaurarlas.

Actualiza también ejemplos/japon-2026-hitos.xlsx con los últimos hitos añadidos.
</commit_message>
<xml_diff>
--- a/ejemplos/japon-2026-hitos.xlsx
+++ b/ejemplos/japon-2026-hitos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L351"/>
+  <dimension ref="A1:L361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9036,6 +9036,256 @@
         </is>
       </c>
     </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>Kurkku Fields</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Hiroshi Nakamura &amp; NAP</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Kisarazu</t>
+        </is>
+      </c>
+      <c r="E352" t="n">
+        <v>2023</v>
+      </c>
+      <c r="L352" t="inlineStr">
+        <is>
+          <t>A · Chiba, ~1 h de Tokio por el Aqua-Line. Granja-parque con la Biblioteca subterránea (Library in the Earth, 2023) y las cabañas Cocoon de Nakamura &amp; NAP; también obras de arte en el paisaje</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>Tanikawa House</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Kazuo Shinohara</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Naganohara</t>
+        </is>
+      </c>
+      <c r="E353" t="n">
+        <v>1974</v>
+      </c>
+      <c r="L353" t="inlineStr">
+        <is>
+          <t>S [R] · Kita-Karuizawa (Gunma). Casa del poeta Tanikawa: el suelo en pendiente de tierra bajo la gran cubierta; obra clave de la tercera etapa de Shinohara. Privada: visitas solo en jornadas concertadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>Shiraiwa Sake Brewery</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Kengo Kuma</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Tateyama</t>
+        </is>
+      </c>
+      <c r="E354" t="n">
+        <v>2021</v>
+      </c>
+      <c r="L354" t="inlineStr">
+        <is>
+          <t>A [R] · Bodega IWA (Richard Geoffroy) en Shiraiwa, falda del Tateyama, Toyama: una sola cubierta negra baja contra los arrozales. Visita con reserva</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>Ebara Hatakeyama Museum of Art</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>New Material Research Laboratory (Hiroshi Sugimoto y Tomoyuki Sakakida) · Taisei</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Tokio</t>
+        </is>
+      </c>
+      <c r="E355" t="n">
+        <v>2024</v>
+      </c>
+      <c r="L355" t="inlineStr">
+        <is>
+          <t>A · Shirokanedai, Tokio. Reabierto en octubre de 2024 tras 4,5 años de obra: edificio principal reformado y ala nueva; jardín con casas de té</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>Pilotis in a Forest</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Go Hasegawa</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Naganohara</t>
+        </is>
+      </c>
+      <c r="E356" t="n">
+        <v>2010</v>
+      </c>
+      <c r="L356" t="inlineStr">
+        <is>
+          <t>S [R] · Kita-Karuizawa (Gunma). Privada; hay que solicitar acceso</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>House in a Forest</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Go Hasegawa</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Karuizawa</t>
+        </is>
+      </c>
+      <c r="E357" t="n">
+        <v>2006</v>
+      </c>
+      <c r="L357" t="inlineStr">
+        <is>
+          <t>S− [R] · Privada; hay que solicitar acceso</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>Roof on a Ridge</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Go Hasegawa</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Nagano</t>
+        </is>
+      </c>
+      <c r="E358" t="n">
+        <v>2020</v>
+      </c>
+      <c r="L358" t="inlineStr">
+        <is>
+          <t>A+ [R] · Nagano, ubicación no pública. Privada; preguntar si coincide geográficamente con la ruta</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>space Un Tokyo</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Go Hasegawa</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Tokio</t>
+        </is>
+      </c>
+      <c r="E359" t="n">
+        <v>2024</v>
+      </c>
+      <c r="L359" t="inlineStr">
+        <is>
+          <t>A/A+ · Aoyama. Pública</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>Sanseido Jimbocho</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Go Hasegawa</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Tokio</t>
+        </is>
+      </c>
+      <c r="E360" t="n">
+        <v>2026</v>
+      </c>
+      <c r="L360" t="inlineStr">
+        <is>
+          <t>A · Jimbōchō. Pública y facilísima</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>Nippon Design Center</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Go Hasegawa</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Tokio</t>
+        </is>
+      </c>
+      <c r="E361" t="n">
+        <v>2012</v>
+      </c>
+      <c r="L361" t="inlineStr">
+        <is>
+          <t>A+ [R] · Ginza. Oficina; acceso académico negociable</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>